<commit_message>
updated crtpal, raf, shelf
</commit_message>
<xml_diff>
--- a/InputData/elec/RAF/Regional Availability Factor.xlsx
+++ b/InputData/elec/RAF/Regional Availability Factor.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\elec\RAF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\RMI\RMI_all_states\KY\elec\RAF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69AC669C-A089-43AC-8C3F-D19C2C3202FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{83D6BAFF-4C7C-458B-B52B-7F9F4706E602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
+    <workbookView xWindow="3510" yWindow="255" windowWidth="12870" windowHeight="17025" activeTab="1" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="53">
   <si>
     <t>Source:</t>
   </si>
@@ -194,6 +194,9 @@
   </si>
   <si>
     <t>hydrogen combined cycle</t>
+  </si>
+  <si>
+    <t>Kentucky</t>
   </si>
 </sst>
 </file>
@@ -245,12 +248,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -565,20 +569,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{667665C7-8A8E-46D9-B686-64BA7741F669}">
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="3">
+        <v>45188</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -586,32 +596,32 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -721,7 +731,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -729,7 +739,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -737,7 +747,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -793,7 +803,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -801,7 +811,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -809,7 +819,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -817,7 +827,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>0.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -825,7 +835,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -833,7 +843,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -841,7 +851,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -849,7 +859,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -857,7 +867,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -865,7 +875,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -873,7 +883,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -881,7 +891,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -889,7 +899,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -897,7 +907,7 @@
         <v>50</v>
       </c>
       <c r="B24">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -905,7 +915,7 @@
         <v>51</v>
       </c>
       <c r="B25">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>